<commit_message>
20250212 introducidos RUN APP desde W y nuevos Excels
</commit_message>
<xml_diff>
--- a/datos/diccionario_EBA_series_df.xlsx
+++ b/datos/diccionario_EBA_series_df.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Apps\bancos_panel\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF10FADD-AE5B-4F6D-B033-EB06A9535D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C90371A-2DB6-4821-B0EE-EAAAEA91D54A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-8700" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="26640" windowHeight="14490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="listado_nombres_Yahoo" sheetId="1" r:id="rId1"/>
@@ -117,33 +117,15 @@
     <t>Ratio de indulgencia</t>
   </si>
   <si>
-    <t>Ratio L/A-depósitos</t>
-  </si>
-  <si>
     <t>Ratio de garantía</t>
   </si>
   <si>
-    <t>Ratio de liquidez</t>
-  </si>
-  <si>
-    <t>Ratio de financiación estable</t>
-  </si>
-  <si>
     <t>ROE</t>
   </si>
   <si>
     <t>ROA</t>
   </si>
   <si>
-    <t>Ingresos netos por intereses</t>
-  </si>
-  <si>
-    <t>Ingresos netos por comisiones</t>
-  </si>
-  <si>
-    <t>Ingresos net por trading</t>
-  </si>
-  <si>
     <t>Margen neto de intereses</t>
   </si>
   <si>
@@ -166,6 +148,24 @@
   </si>
   <si>
     <t>Ratio de eficiencia</t>
+  </si>
+  <si>
+    <t>LCR</t>
+  </si>
+  <si>
+    <t>Loan-to-Deposit ratio</t>
+  </si>
+  <si>
+    <t>% de ingresos por comisiones</t>
+  </si>
+  <si>
+    <t>% de ingresos trading</t>
+  </si>
+  <si>
+    <t>NSFR</t>
+  </si>
+  <si>
+    <t>% de ingresos netos de intereses</t>
   </si>
 </sst>
 </file>
@@ -606,21 +606,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="124.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="124.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -628,7 +628,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -636,7 +636,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -644,7 +644,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -652,95 +652,95 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -748,44 +748,44 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -797,15 +797,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010025A34F53D094394FB21F9DBA6BFE7698" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="e7ecd460bafe359a3215e5e4c7378472">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e3a2ec7d-e900-4ee0-8b1e-fac67f483317" xmlns:ns3="6cb3014e-c15e-4453-8639-5b8772973515" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="be8bf92af2a4fb1c1e1376e9b2342f6b" ns2:_="" ns3:_="">
     <xsd:import namespace="e3a2ec7d-e900-4ee0-8b1e-fac67f483317"/>
@@ -1034,15 +1025,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB2D8C0E-0D2C-4690-9BA9-66778D4103C3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B631D2E4-1361-44A9-B26B-72C624D3CD94}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1059,4 +1051,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB2D8C0E-0D2C-4690-9BA9-66778D4103C3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>